<commit_message>
feat(esg): mức độ công bố ESG theo trụ cột E/S/G từ file Excel
- Đọc sheet ESG_ChiTieu (32 chỉ tiêu ESG công bố 2024) → esg_indicators.json
  → getEsgIndicators(); thêm cột unit, rule (Gốc / Chia DT) vào sheet
- Thẻ "Điểm ESG" ở Cổng 1: thực hành áp dụng và số liệu định lượng đã công
  bố theo E/S/G so với trung bình 4 DN; tab chi tiết từng chỉ tiêu với hạng
  trong nhóm theo chiều tốt. Chỉ đếm trên dữ liệu thật, không chấm điểm
- Không xếp hạng chỉ tiêu số tuyệt đối phụ thuộc quy mô (tránh "DN nhỏ
  phát thải ít = tốt"); radar điểm trụ cột chỉ hiện khi có điểm thật
- Badge tẩy xanh "chưa đánh giá"; tóm tắt mức độ công bố trong báo cáo
- Unit test + e2e; cập nhật DATA, UI_DESIGN, TECH_STACK
- Bỏ qua file khoá LibreOffice/Excel trong git

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/QuantumRegTech_Data.xlsx
+++ b/data/QuantumRegTech_Data.xlsx
@@ -152,10 +152,31 @@
     <author>Author</author>
   </authors>
   <commentList>
+    <comment ref="B1" authorId="0">
+      <text>
+        <r>
+          <t>Tên chỉ tiêu hiển thị trên UI (đơn vị ở cột unit)</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="E1" authorId="0">
       <text>
         <r>
           <t>0 = chỉ tiêu bị loại</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0">
+      <text>
+        <r>
+          <t>Đơn vị hiển thị của chỉ tiêu định lượng (Num)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0">
+      <text>
+        <r>
+          <t>Gốc = dùng trực tiếp; Chia DT = số tuyệt đối phải chia doanh thu khi so sánh (quy ước AQ_Input)</t>
         </r>
       </text>
     </comment>
@@ -514,7 +535,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="307">
   <si>
     <t>QuantumRegTech – FILE DỮ LIỆU CHO UI (nguồn dữ liệu duy nhất của app)</t>
   </si>
@@ -558,7 +579,7 @@
     <t>ESG – điểm ESGi &amp; trụ cột · ESG_Evidence – bằng chứng tẩy xanh · OSINT – sự kiện · Portfolio – tỷ trọng · Portfolio_Summary – lợi nhuận danh mục · Scenarios – kịch bản slider</t>
   </si>
   <si>
-    <t>QUBO_Matrix – ma trận Q (để trống) · Private_Sample – kết quả mẫu Cổng 2 · ESG_ChiTieu – chỉ tiêu ESG thô 2024 (tham khảo, app chưa đọc) · Cho_xac_nhan – việc cần nhóm quyết định</t>
+    <t>QUBO_Matrix – ma trận Q (để trống) · Private_Sample – kết quả mẫu Cổng 2 · ESG_ChiTieu – 32 chỉ tiêu ESG công bố 2024 (app hiển thị mức độ công bố ở Cổng 1) · Cho_xac_nhan – việc cần nhóm quyết định</t>
   </si>
   <si>
     <t>key</t>
@@ -1104,10 +1125,16 @@
     <t>TH</t>
   </si>
   <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>rule</t>
+  </si>
+  <si>
     <t>E_01</t>
   </si>
   <si>
-    <t>Tổng phát thải khí nhà kính Scope 1 &amp; 2 (tấn CO2e)</t>
+    <t>Tổng phát thải khí nhà kính Scope 1 &amp; 2</t>
   </si>
   <si>
     <t>Num</t>
@@ -1116,10 +1143,19 @@
     <t>(-)</t>
   </si>
   <si>
+    <t>tấn CO2e</t>
+  </si>
+  <si>
+    <t>Gốc</t>
+  </si>
+  <si>
     <t>E_02</t>
   </si>
   <si>
-    <t>Cường độ phát thải (tấn CO2e/tỷ đồng doanh thu)</t>
+    <t>Cường độ phát thải</t>
+  </si>
+  <si>
+    <t>tấn CO2e/tỷ đồng DT</t>
   </si>
   <si>
     <t>E_03</t>
@@ -1149,25 +1185,37 @@
     <t>E_06</t>
   </si>
   <si>
-    <t>Tổng lượng nước tiêu thụ (m3) – code tự chia doanh thu</t>
+    <t>Tổng lượng nước tiêu thụ</t>
+  </si>
+  <si>
+    <t>m³</t>
+  </si>
+  <si>
+    <t>Chia DT</t>
   </si>
   <si>
     <t>E_07</t>
   </si>
   <si>
-    <t>Tỷ lệ nước tái sử dụng/tuần hoàn (%)</t>
+    <t>Tỷ lệ nước tái sử dụng/tuần hoàn</t>
+  </si>
+  <si>
+    <t>%</t>
   </si>
   <si>
     <t>E_08</t>
   </si>
   <si>
-    <t>Tổng năng lượng tiêu thụ (GJ) – code tự chia doanh thu</t>
+    <t>Tổng năng lượng tiêu thụ</t>
+  </si>
+  <si>
+    <t>GJ</t>
   </si>
   <si>
     <t>E_09</t>
   </si>
   <si>
-    <t>Tỷ lệ năng lượng tái tạo (%)</t>
+    <t>Tỷ lệ năng lượng tái tạo</t>
   </si>
   <si>
     <t>E_10</t>
@@ -1179,7 +1227,7 @@
     <t>E_11</t>
   </si>
   <si>
-    <t>Chi đầu tư cho R&amp;D/Công nghệ xanh (VND)</t>
+    <t>Chi đầu tư cho R&amp;D/Công nghệ xanh</t>
   </si>
   <si>
     <t>E_12</t>
@@ -1194,10 +1242,13 @@
     <t>Tổng số nhân viên (Quy mô lao động)</t>
   </si>
   <si>
+    <t>người</t>
+  </si>
+  <si>
     <t>S_02</t>
   </si>
   <si>
-    <t>Tỷ lệ nữ giới trong ban quản lý cấp cao ( ban điều hành) (%)</t>
+    <t>Tỷ lệ nữ giới trong ban quản lý cấp cao (ban điều hành)</t>
   </si>
   <si>
     <t>S_03</t>
@@ -1206,6 +1257,9 @@
     <t>Số giờ đào tạo trung bình/nhân viên</t>
   </si>
   <si>
+    <t>giờ/người</t>
+  </si>
+  <si>
     <t>S_04</t>
   </si>
   <si>
@@ -1215,13 +1269,13 @@
     <t>S_05</t>
   </si>
   <si>
-    <t xml:space="preserve">Hoạt động, chính sách, chi phí đầu tư và sự tuân thủ cho sự an toàn của lao động </t>
+    <t>Hoạt động, chính sách, chi phí đầu tư và sự tuân thủ cho sự an toàn của lao động</t>
   </si>
   <si>
     <t>S_06</t>
   </si>
   <si>
-    <t xml:space="preserve">Công bố về tai nạn lao động </t>
+    <t>Công bố về tai nạn lao động</t>
   </si>
   <si>
     <t>S_07</t>
@@ -1239,7 +1293,10 @@
     <t>S_09</t>
   </si>
   <si>
-    <t>Tổng ngân sách đóng góp xã hội (tỷ đồng) – code tự chia doanh thu</t>
+    <t>Tổng ngân sách đóng góp xã hội</t>
+  </si>
+  <si>
+    <t>tỷ đồng</t>
   </si>
   <si>
     <t>S_10</t>
@@ -1272,10 +1329,13 @@
     <t>Quy mô Hội đồng quản trị (HĐQT)</t>
   </si>
   <si>
+    <t>thành viên</t>
+  </si>
+  <si>
     <t>G_02</t>
   </si>
   <si>
-    <t>Tỷ lệ thành viên HĐQT độc lập (%)</t>
+    <t>Tỷ lệ thành viên HĐQT độc lập</t>
   </si>
   <si>
     <t>G_03</t>
@@ -2615,7 +2675,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -2623,9 +2683,11 @@
     <col min="3" max="3" width="6" customWidth="1"/>
     <col min="4" max="5" width="5" customWidth="1"/>
     <col min="6" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="12" max="12" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>192</v>
       </c>
@@ -2656,19 +2718,25 @@
       <c r="J1" s="3" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -2688,19 +2756,25 @@
       <c r="J2">
         <v>339425</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K2" t="s">
+        <v>202</v>
+      </c>
+      <c r="L2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B3" t="s">
+        <v>205</v>
+      </c>
+      <c r="C3" t="s">
         <v>200</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>201</v>
-      </c>
-      <c r="C3" t="s">
-        <v>198</v>
-      </c>
-      <c r="D3" t="s">
-        <v>199</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2717,19 +2791,25 @@
       <c r="I3">
         <v>2.34</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K3" t="s">
+        <v>206</v>
+      </c>
+      <c r="L3" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="B4" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="C4" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D4" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2749,19 +2829,22 @@
       <c r="J4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L4" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="B5" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C5" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D5" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2781,19 +2864,22 @@
       <c r="J5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L5" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B6" t="s">
+        <v>214</v>
+      </c>
+      <c r="C6" t="s">
         <v>209</v>
       </c>
-      <c r="C6" t="s">
-        <v>204</v>
-      </c>
       <c r="D6" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2813,19 +2899,22 @@
       <c r="J6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L6" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="B7" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="C7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D7" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2842,19 +2931,25 @@
       <c r="J7">
         <v>6394459</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K7" t="s">
+        <v>217</v>
+      </c>
+      <c r="L7" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="B8" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="C8" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D8" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2871,19 +2966,25 @@
       <c r="J8">
         <v>37.1</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K8" t="s">
+        <v>221</v>
+      </c>
+      <c r="L8" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="B9" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="C9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D9" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2900,19 +3001,25 @@
       <c r="J9">
         <v>1020968</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K9" t="s">
+        <v>224</v>
+      </c>
+      <c r="L9" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="B10" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="C10" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D10" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2929,19 +3036,25 @@
       <c r="J10">
         <v>15.23</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K10" t="s">
+        <v>221</v>
+      </c>
+      <c r="L10" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="B11" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="C11" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D11" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2961,19 +3074,22 @@
       <c r="J11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L11" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="B12" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="C12" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D12" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2993,19 +3109,22 @@
       <c r="J12">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L12" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="B13" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="C13" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D13" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -3025,19 +3144,22 @@
       <c r="J13">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L13" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="B14" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="C14" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D14" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -3057,19 +3179,25 @@
       <c r="J14">
         <v>10000</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K14" t="s">
+        <v>235</v>
+      </c>
+      <c r="L14" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="B15" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="C15" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D15" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -3089,19 +3217,25 @@
       <c r="J15">
         <v>31</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K15" t="s">
+        <v>221</v>
+      </c>
+      <c r="L15" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="B16" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="C16" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D16" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -3118,19 +3252,25 @@
       <c r="J16">
         <v>33.4</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K16" t="s">
+        <v>240</v>
+      </c>
+      <c r="L16" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
       <c r="B17" t="s">
-        <v>231</v>
+        <v>242</v>
       </c>
       <c r="C17" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D17" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -3150,19 +3290,22 @@
       <c r="J17">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L17" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>232</v>
+        <v>243</v>
       </c>
       <c r="B18" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="C18" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D18" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -3182,19 +3325,22 @@
       <c r="J18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L18" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
       <c r="B19" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="C19" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D19" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -3214,19 +3360,22 @@
       <c r="J19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L19" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="B20" t="s">
-        <v>237</v>
+        <v>248</v>
       </c>
       <c r="C20" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D20" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -3246,19 +3395,22 @@
       <c r="J20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L20" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
       <c r="B21" t="s">
-        <v>239</v>
+        <v>250</v>
       </c>
       <c r="C21" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D21" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -3278,19 +3430,22 @@
       <c r="J21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L21" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="B22" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
       <c r="C22" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D22" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -3310,19 +3465,25 @@
       <c r="J22">
         <v>95.2</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K22" t="s">
+        <v>253</v>
+      </c>
+      <c r="L22" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="B23" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="C23" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D23" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -3342,19 +3503,22 @@
       <c r="J23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L23" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="B24" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="C24" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D24" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -3374,19 +3538,22 @@
       <c r="J24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L24" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="B25" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="C25" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D25" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -3406,19 +3573,22 @@
       <c r="J25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L25" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="B26" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="C26" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D26" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -3438,19 +3608,22 @@
       <c r="J26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L26" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="B27" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="C27" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D27" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -3467,19 +3640,25 @@
       <c r="I27">
         <v>8</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K27" t="s">
+        <v>264</v>
+      </c>
+      <c r="L27" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="B28" t="s">
-        <v>253</v>
+        <v>266</v>
       </c>
       <c r="C28" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D28" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -3496,19 +3675,25 @@
       <c r="I28">
         <v>25</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K28" t="s">
+        <v>221</v>
+      </c>
+      <c r="L28" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="B29" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="C29" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D29" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -3528,19 +3713,22 @@
       <c r="J29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L29" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
       <c r="B30" t="s">
-        <v>257</v>
+        <v>270</v>
       </c>
       <c r="C30" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D30" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -3557,19 +3745,25 @@
       <c r="I30">
         <v>37.5</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K30" t="s">
+        <v>221</v>
+      </c>
+      <c r="L30" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="B31" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C31" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D31" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -3589,19 +3783,22 @@
       <c r="J31">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L31" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="B32" t="s">
-        <v>261</v>
+        <v>274</v>
       </c>
       <c r="C32" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D32" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E32">
         <v>1</v>
@@ -3621,19 +3818,22 @@
       <c r="J32">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L32" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
       <c r="B33" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
       <c r="C33" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D33" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -3652,6 +3852,9 @@
       </c>
       <c r="J33">
         <v>0</v>
+      </c>
+      <c r="L33" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -3678,16 +3881,16 @@
         <v>137</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>264</v>
+        <v>277</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>265</v>
+        <v>278</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>267</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="23" customFormat="1" x14ac:dyDescent="0.25">
@@ -3695,16 +3898,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>268</v>
+        <v>281</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>269</v>
+        <v>282</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>270</v>
+        <v>283</v>
       </c>
       <c r="E2" s="24" t="s">
-        <v>271</v>
+        <v>284</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="23" customFormat="1" x14ac:dyDescent="0.25">
@@ -3712,16 +3915,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>272</v>
+        <v>285</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>273</v>
+        <v>286</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>274</v>
+        <v>287</v>
       </c>
       <c r="E3" s="24" t="s">
-        <v>271</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="23" customFormat="1" x14ac:dyDescent="0.25">
@@ -3729,16 +3932,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>275</v>
+        <v>288</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>271</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="23" customFormat="1" x14ac:dyDescent="0.25">
@@ -3746,16 +3949,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>278</v>
+        <v>291</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>279</v>
+        <v>292</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>271</v>
+        <v>284</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="23" customFormat="1" x14ac:dyDescent="0.25">
@@ -3763,16 +3966,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>281</v>
+        <v>294</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>271</v>
+        <v>284</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="23" customFormat="1" x14ac:dyDescent="0.25">
@@ -3780,16 +3983,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="23" t="s">
+        <v>297</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>298</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>299</v>
+      </c>
+      <c r="E7" s="24" t="s">
         <v>284</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>285</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>286</v>
-      </c>
-      <c r="E7" s="24" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="23" customFormat="1" x14ac:dyDescent="0.25">
@@ -3797,16 +4000,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>288</v>
+        <v>301</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>289</v>
+        <v>302</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="23" customFormat="1" x14ac:dyDescent="0.25">
@@ -3814,21 +4017,21 @@
         <v>8</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>291</v>
+        <v>304</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>292</v>
+        <v>305</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>293</v>
+        <v>306</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 

</xml_diff>